<commit_message>
Enrich competitor analysis with full seller ranking (26165 sellers)
- Add 'Рынок_ТОП' sheet: category top-13 (Ozon, RU mass-brands, clones, us)
- Add 'Клоны_Celimax' sheet: all three Celimax resellers rank ahead of us
  (LIFECOSM #7, MASKSHOP #24, THE:BO #32 vs KOREADOM #99)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0153XBqtvJYtRAKHdw3RmMsz
</commit_message>
<xml_diff>
--- a/outputs/ozon_competitors/ozon_competitor_analysis_2026-09-29.xlsx
+++ b/outputs/ozon_competitors/ozon_competitor_analysis_2026-09-29.xlsx
@@ -8,11 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="Итоги" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Продавцы" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Тонер_Celimax" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="LIFECOSM_товары" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Категории" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Бренды" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Рынок_ТОП" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Клоны_Celimax" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Продавцы" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Тонер_Celimax" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="LIFECOSM_товары" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Категории" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Бренды" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -45,7 +47,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -65,6 +67,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -94,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -121,6 +128,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -702,6 +715,697 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Категория «Косметика для ухода» — топ продавцов из 26 165</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>Позиция</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>Продавец</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>Заказано, ₽</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>Заказано, шт</t>
+        </is>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>Ср.цена, ₽</t>
+        </is>
+      </c>
+      <c r="F3" s="14" t="inlineStr">
+        <is>
+          <t>Брендов</t>
+        </is>
+      </c>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>Кластеров</t>
+        </is>
+      </c>
+      <c r="H3" s="14" t="inlineStr">
+        <is>
+          <t>Выкуп</t>
+        </is>
+      </c>
+      <c r="I3" s="14" t="inlineStr">
+        <is>
+          <t>Тип игрока</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Ozon (сам маркетплейс)</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>316368720</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>472267</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>670</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>158</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="H4" s="8" t="n">
+        <v>0.912</v>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Площадка</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Гельтек</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>209646007</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>197032</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>1064</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>0.872</v>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>RU проф-бренд</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>ARAVIA</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>177139982</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>478372</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>370</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="H6" s="8" t="n">
+        <v>0.917</v>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>RU масс-бренд</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>MIXIT</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>160068559</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>342214</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>468</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>0.902</v>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>RU масс-бренд</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>VOIS</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>139608642</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>369139</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>378</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="H8" s="8" t="n">
+        <v>0.858</v>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>RU масс-бренд</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>NAOS</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>81948343</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>55044</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>1489</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>Импорт (Bioderma)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>LIFECOSM</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>76072289</v>
+      </c>
+      <c r="D10" s="16" t="n">
+        <v>59478</v>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>1279</v>
+      </c>
+      <c r="F10" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="G10" s="15" t="n">
+        <v>29</v>
+      </c>
+      <c r="H10" s="17" t="n">
+        <v>0.8129999999999999</v>
+      </c>
+      <c r="I10" s="15" t="inlineStr">
+        <is>
+          <t>КЛОН Celimax</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Cream.Shop</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>75679831</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>52484</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>1442</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>0.848</v>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>Корейский селлер</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>GRACEFACE</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>70472067</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>203023</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>347</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="H12" s="8" t="n">
+        <v>0.9330000000000001</v>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>RU масс-бренд</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>РИВ ГОШ</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>65098674</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>98862</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>658</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>204</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="H13" s="8" t="n">
+        <v>0.888</v>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>Ритейл-сеть</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>MASKSHOP.RU</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="n">
+        <v>30821788</v>
+      </c>
+      <c r="D14" s="16" t="n">
+        <v>21935</v>
+      </c>
+      <c r="E14" s="16" t="n">
+        <v>1405</v>
+      </c>
+      <c r="F14" s="15" t="n"/>
+      <c r="G14" s="15" t="n">
+        <v>29</v>
+      </c>
+      <c r="H14" s="15" t="n"/>
+      <c r="I14" s="15" t="inlineStr">
+        <is>
+          <t>КЛОН Celimax</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="n">
+        <v>32</v>
+      </c>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>THE:BO</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="n">
+        <v>20956111</v>
+      </c>
+      <c r="D15" s="16" t="n">
+        <v>19431</v>
+      </c>
+      <c r="E15" s="16" t="n">
+        <v>1079</v>
+      </c>
+      <c r="F15" s="15" t="n"/>
+      <c r="G15" s="15" t="n">
+        <v>29</v>
+      </c>
+      <c r="H15" s="15" t="n"/>
+      <c r="I15" s="15" t="inlineStr">
+        <is>
+          <t>КЛОН Celimax</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>99</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>KOREADOM (мы)</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="n">
+        <v>6103290</v>
+      </c>
+      <c r="D16" s="18" t="n">
+        <v>5203</v>
+      </c>
+      <c r="E16" s="18" t="n">
+        <v>1173</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="H16" s="19" t="n">
+        <v>0.862</v>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>МЫ</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Верх категории — площадка Ozon и российские масс-бренды (350–670 ₽, объём миллионами штук) — другой сегмент. Наш прямой ориентир — корейские селлеры каталога Celimax (жёлтые).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A18:I19"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Продавцы того же каталога Celimax — все три обгоняют нас</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>Продавец</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>Позиция</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>Заказано, ₽</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>Заказано, шт</t>
+        </is>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>Кластеров</t>
+        </is>
+      </c>
+      <c r="F3" s="14" t="inlineStr">
+        <is>
+          <t>Доля категории</t>
+        </is>
+      </c>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>Во сколько раз &gt; нас (₽)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>LIFECOSM</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="C4" s="16" t="n">
+        <v>76072289</v>
+      </c>
+      <c r="D4" s="16" t="n">
+        <v>59478</v>
+      </c>
+      <c r="E4" s="15" t="n">
+        <v>29</v>
+      </c>
+      <c r="F4" s="17" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="G4" s="15" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>MASKSHOP.RU</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="C5" s="16" t="n">
+        <v>30821788</v>
+      </c>
+      <c r="D5" s="16" t="n">
+        <v>21935</v>
+      </c>
+      <c r="E5" s="15" t="n">
+        <v>29</v>
+      </c>
+      <c r="F5" s="17" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="G5" s="15" t="n">
+        <v>5.1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>THE:BO</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="n">
+        <v>32</v>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>20956111</v>
+      </c>
+      <c r="D6" s="16" t="n">
+        <v>19431</v>
+      </c>
+      <c r="E6" s="15" t="n">
+        <v>29</v>
+      </c>
+      <c r="F6" s="17" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="G6" s="15" t="n">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>KOREADOM (мы)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>99</v>
+      </c>
+      <c r="C7" s="18" t="n">
+        <v>6103290</v>
+      </c>
+      <c r="D7" s="18" t="n">
+        <v>5203</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="F7" s="19" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Все клоны держат 29 кластеров против наших 27 и имеют больший сток. Вывод неизменен: обгон — через наличие топ-SKU и расширение каталога, не через цену.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A9:G10"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -841,7 +1545,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -993,7 +1697,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1373,7 +2077,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1602,7 +2306,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>